<commit_message>
Add desktop edition (pywebview) with downloads fix and asset-delete crash fix
</commit_message>
<xml_diff>
--- a/static/templates/aps-employees-template.xlsx
+++ b/static/templates/aps-employees-template.xlsx
@@ -519,12 +519,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mohammad Shahriyar Hasan</t>
+          <t>Jane Example Doe</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>M3146</t>
+          <t>EMP-1025</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>01712-345678</t>
+          <t>01700-000000</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>employee_id   — unique ID (e.g. M3146). Required. Duplicates are skipped.</t>
+          <t>employee_id   — unique ID (e.g. EMP-1025). Required. Duplicates are skipped.</t>
         </is>
       </c>
     </row>

</xml_diff>